<commit_message>
Release guided workload contract
</commit_message>
<xml_diff>
--- a/artifacts/AI_Build_Crew_Agentic_AI_PRD_COST_CONTRACT.xlsx
+++ b/artifacts/AI_Build_Crew_Agentic_AI_PRD_COST_CONTRACT.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rc67e6e331dc343b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R4cefe2b729024d87"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,9 +13,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
-    <x:numFmt numFmtId="201" formatCode="mmmm d, yyyy"/>
   </x:numFmts>
   <x:fonts count="11">
     <x:font>
@@ -181,7 +180,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -304,9 +303,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -546,7 +542,7 @@
         <x:v>Your Name:</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Christopher Ansted</x:v>
+        <x:v>Charles Tansted</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
@@ -572,7 +568,7 @@
         <x:v>Workflow / Project Choice:</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>A prompt-first planning workflow that helps a product builder turn an incomplete AI idea into a visible workload, a low/likely/high cost-per-completed-task range, a policy-eligible starting point, and a human-owned decision.</x:v>
+        <x:v>A prompt-first decision workflow where a product builder turns an incomplete AI idea into a confirmed workload, a deterministic model starting point, a low/likely/high cost-per-completed-task range, separate cost evaluation/audit/governance evidence, and a human-owned decision.</x:v>
       </x:c>
       <x:c r="C5" s="1"/>
       <x:c r="D5" s="1"/>
@@ -584,7 +580,7 @@
       <x:c r="A6" s="6" t="str">
         <x:v>Date:</x:v>
       </x:c>
-      <x:c r="B6" s="49" t="n">
+      <x:c r="B6" s="10" t="n">
         <x:v>46243.708333333336</x:v>
       </x:c>
       <x:c r="C6" s="1"/>
@@ -609,10 +605,10 @@
       <x:c r="B8" s="15" t="str">
         <x:v>Agentic AI PRD</x:v>
       </x:c>
-      <x:c r="C8" s="15"/>
-      <x:c r="D8" s="15"/>
-      <x:c r="E8" s="15"/>
-      <x:c r="F8" s="15"/>
+      <x:c r="C8" s="15" t="str"/>
+      <x:c r="D8" s="15" t="str"/>
+      <x:c r="E8" s="15" t="str"/>
+      <x:c r="F8" s="15" t="str"/>
       <x:c r="G8" s="15" t="str">
         <x:v>Faculty Feedback</x:v>
       </x:c>
@@ -657,12 +653,12 @@
         <x:v>Who is the specific user this agent helps?</x:v>
       </x:c>
       <x:c r="F10" s="31" t="str">
-        <x:v>The first user is a product person building an AI-powered application, agent, or tool without a dedicated AI architect or FinOps partner. They understand the user problem and business constraints, but may not know model names, token math, caching, or provider pricing. The beachhead is first-time AI product builders and small product teams that need a decision they can explain.</x:v>
-      </x:c>
-      <x:c r="G10" s="31"/>
+        <x:v>The first persona is an early-stage product builder or product manager with a real AI product idea, limited AI architecture or FinOps support, and responsibility for a go/no-go build decision. The initial beachhead is small product teams that must choose a model starting point, forecast completed-task cost, and defend the decision before committing engineering time or provider spend.</x:v>
+      </x:c>
+      <x:c r="G10" s="31" t="str"/>
     </x:row>
     <x:row r="11" ht="88" customHeight="1">
-      <x:c r="A11" s="20"/>
+      <x:c r="A11" s="20" t="str"/>
       <x:c r="B11" s="20" t="str">
         <x:v>Project choice</x:v>
       </x:c>
@@ -676,12 +672,12 @@
         <x:v>What recurring workflow are you improving? Write the current workflow in plain text.</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>The recurring workflow is the decision before the build: define what the AI must do, turn the idea into a workload, estimate model-usage cost, compare eligible options, surface risk and missing evidence, and decide what to test or build next.</x:v>
-      </x:c>
-      <x:c r="G11" s="26"/>
+        <x:v>The recurring workflow is pre-build model selection and cost planning. The user turns a rough AI product idea into a workload description, researches candidate models and pricing, estimates token and workflow usage, compares cost/quality/latency/risk tradeoffs, identifies design optimizations, and prepares a decision for review.</x:v>
+      </x:c>
+      <x:c r="G11" s="26" t="str"/>
     </x:row>
     <x:row r="12" ht="88" customHeight="1">
-      <x:c r="A12" s="20"/>
+      <x:c r="A12" s="20" t="str"/>
       <x:c r="B12" s="20" t="str">
         <x:v>Project choice</x:v>
       </x:c>
@@ -695,12 +691,12 @@
         <x:v>What event starts the workflow?</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>The workflow starts when someone has an AI product idea, feature, agent, or architecture choice and needs a model starting point and cost range before committing engineering time, budget, or approval.</x:v>
-      </x:c>
-      <x:c r="G12" s="26"/>
+        <x:v>The workflow starts when the user has an AI product idea, feature, agent, prompt workflow, or architecture decision and must choose a model and estimate cost before committing engineering effort or seeking approval.</x:v>
+      </x:c>
+      <x:c r="G12" s="26" t="str"/>
     </x:row>
     <x:row r="13" ht="88" customHeight="1">
-      <x:c r="A13" s="20"/>
+      <x:c r="A13" s="20" t="str"/>
       <x:c r="B13" s="20" t="str">
         <x:v>Current state</x:v>
       </x:c>
@@ -714,12 +710,12 @@
         <x:v>List the current process as numbered text steps. Do not link to a process map.</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>1. Describe the idea in plain language. 2. Search provider pricing and model pages. 3. Translate different price units and capability claims. 4. Guess volume, input size, output tokens, cache, and model calls. 5. Lock one output number and one call across unlike models. 6. Compare monthly totals in notes or a spreadsheet. 7. Discover later that retries, checkers, and longer reasoning output changed the unit cost. 8. Rework and re-explain the choice.</x:v>
-      </x:c>
-      <x:c r="G13" s="26"/>
+        <x:v>1. Describe the product idea informally. 2. Search provider pages and third-party comparisons. 3. Try to understand model capabilities and price units. 4. Guess input/output token volumes, number of calls, context, tools, retrieval, and loops. 5. Compare candidates manually, often in notes or a spreadsheet. 6. Select a familiar or premium model when evidence is unclear. 7. Revise the estimate when assumptions or prices change. 8. Explain the choice to reviewers without a consistent decision record.</x:v>
+      </x:c>
+      <x:c r="G13" s="26" t="str"/>
     </x:row>
     <x:row r="14" ht="88" customHeight="1">
-      <x:c r="A14" s="20"/>
+      <x:c r="A14" s="20" t="str"/>
       <x:c r="B14" s="20" t="str">
         <x:v>Problem</x:v>
       </x:c>
@@ -733,12 +729,12 @@
         <x:v>Where does the workflow slow down, fail, create rework, or frustrate the user?</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>The work breaks in four places. The user may not know what to estimate. Provider rates and fee coverage differ and change. Output length and retries vary by model and run. Public benchmarks do not prove fit for the real workload. The result is hidden assumptions, false precision, repeated work, and a monthly total that can understate cost per completed task.</x:v>
-      </x:c>
-      <x:c r="G14" s="26"/>
+        <x:v>Early-stage builders are forced to choose models before they understand the workload shape. Provider pricing is fragmented, while output length, retry behavior, checker calls, and uncovered fees vary by model. The result is false precision, underbudgeted completed-task cost, rework, and model decisions that cannot be reproduced or defended.</x:v>
+      </x:c>
+      <x:c r="G14" s="26" t="str"/>
     </x:row>
     <x:row r="15" ht="88" customHeight="1">
-      <x:c r="A15" s="20"/>
+      <x:c r="A15" s="20" t="str"/>
       <x:c r="B15" s="20" t="str">
         <x:v>Opportunity</x:v>
       </x:c>
@@ -752,12 +748,12 @@
         <x:v>What should the agent help with, and why is an agent a better fit than a static AI feature?</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>AI Build Crew should guide only as far as needed, keep assumptions visible, apply dated prices, reject user-entered output tokens, use model-specific low/likely/high output and retry profiles, include primary and checker steps, rank by cost per completed task, independently check the ledger, and return the decision to a human.</x:v>
-      </x:c>
-      <x:c r="G15" s="26"/>
+        <x:v>The agent should interview the user about intent and constraints, detect missing assumptions, retrieve a normalized model catalog, calculate scenarios, filter ineligible models, compare tradeoffs, recommend tuning, and produce a reviewable decision brief. An agent is a better fit than a static calculator because the required questions and recommendations change based on the workload, risk, missing information, and previous answers.</x:v>
+      </x:c>
+      <x:c r="G15" s="26" t="str"/>
     </x:row>
     <x:row r="16" ht="88" customHeight="1">
-      <x:c r="A16" s="20"/>
+      <x:c r="A16" s="20" t="str"/>
       <x:c r="B16" s="20" t="str">
         <x:v>Data</x:v>
       </x:c>
@@ -771,12 +767,12 @@
         <x:v>What synthetic data, policies, examples, or cases will you create so the project is safe to build and demo?</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>Use fictional workloads only: a support classifier, document summary, coding assistant, RAG question-answering flow, image task, high-risk medical draft, excessive agent loop, missing-data case, stale catalog, and no-eligible-model case. Use versioned policy rules and dated catalog snapshots. No customer, employer, secret, proprietary, or protected health data is needed for the build or demo.</x:v>
-      </x:c>
-      <x:c r="G16" s="26"/>
+        <x:v>Create a synthetic model catalog with clearly marked sample prices and capabilities for development, plus at least eight fictional workload plans: customer-support classifier, document summarizer, code assistant, RAG Q&amp;A, image extraction, high-risk medical draft, agent with excessive loops, and a workload with missing data. Create policy rules for risk, required human review, stale pricing, missing capability evidence, and unsupported modalities. No customer, employer, medical, or proprietary data is required.</x:v>
+      </x:c>
+      <x:c r="G16" s="26" t="str"/>
     </x:row>
     <x:row r="17" ht="88" customHeight="1">
-      <x:c r="A17" s="20"/>
+      <x:c r="A17" s="20" t="str"/>
       <x:c r="B17" s="20" t="str">
         <x:v>Safety</x:v>
       </x:c>
@@ -790,12 +786,12 @@
         <x:v>What is the agent not allowed to do? When must a human approve, edit, reject, or escalate?</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>The system cannot invent prices or capabilities, claim a universally best model, purchase access, deploy traffic, approve regulated or high-risk use, or treat unknown data as safe. A human must confirm assumptions and own the final choice. High-risk, regulated, sensitive, stale, unsupported, or failed-check cases require review or block the decision.</x:v>
-      </x:c>
-      <x:c r="G17" s="26"/>
+        <x:v>The agent cannot claim a universally best model, invent price or capability facts, purchase or provision access, deploy a workload, approve a regulated or high-risk use case, or use protected data. A human must approve the final model decision, review any high-risk or low-confidence recommendation, accept or edit workload assumptions, and record the reason for overriding the recommendation.</x:v>
+      </x:c>
+      <x:c r="G17" s="26" t="str"/>
     </x:row>
     <x:row r="18" ht="88" customHeight="1">
-      <x:c r="A18" s="20"/>
+      <x:c r="A18" s="20" t="str"/>
       <x:c r="B18" s="20" t="str">
         <x:v>Measurement</x:v>
       </x:c>
@@ -809,12 +805,12 @@
         <x:v>What is one practical metric that would show the agent is useful?</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>Primary metric: a first-time AI product builder reaches a labeled cost-per-completed-task range in under three minutes and explains the recommendation plus one alternative tradeoff. Release control: every cost-contract, deterministic, and governance case passes, and no unsafe or unknown case is marked ready without review.</x:v>
-      </x:c>
-      <x:c r="G18" s="26"/>
+        <x:v>Primary metric: a first-time builder can produce a first estimate in under three minutes and explain the recommendation, one cost assumption, and one alternative tradeoff. Release quality requires every deterministic cost, evaluation, audit, and governance regression case to pass; high-risk, unknown-safety, or unsupported multi-format work can never be marked ready without review.</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="str"/>
     </x:row>
     <x:row r="19" ht="88" customHeight="1">
-      <x:c r="A19" s="20"/>
+      <x:c r="A19" s="20" t="str"/>
       <x:c r="B19" s="20" t="str">
         <x:v>Demo</x:v>
       </x:c>
@@ -828,9 +824,9 @@
         <x:v>What will the demo visibly show from input to agent work to human review?</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>The reviewer sees the full loop: describe an idea, confirm result shape and workflow steps, calculate low/likely/high cost per completed task from model-owned behavior profiles, independently recompute the ledger, inspect the policy-eligible starting point and alternatives, review governance findings, and leave the final decision with the human.</x:v>
-      </x:c>
-      <x:c r="G19" s="26"/>
+        <x:v>The demo opens by asking what the builder is considering building. The builder chooses a guided, known-usage, or safe-example route. The workflow records confirmed and assumed fields, recommends a visible starting number of primary and checker steps when the user does not know, calculates low/likely/high cost per completed task, filters candidates that cannot support every selected format, and explains what would change the model result. Cost Evaluation, Audit, and Governance run against the frozen result before the Human Decision Gate becomes available.</x:v>
+      </x:c>
+      <x:c r="G19" s="26" t="str"/>
     </x:row>
     <x:row r="20" ht="88" customHeight="1">
       <x:c r="A20" s="36" t="str">
@@ -849,12 +845,12 @@
         <x:v>What job is the agent being hired to do?</x:v>
       </x:c>
       <x:c r="F20" s="34" t="str">
-        <x:v>Help a product builder answer: What could this AI idea cost to run, which model is a defensible starting point, where is the estimate uncertain, and what changes if I choose differently?</x:v>
-      </x:c>
-      <x:c r="G20" s="34"/>
+        <x:v>WHEN I am deciding whether and how to build an AI-powered product, agent, or workflow—but I do not yet know the model architecture or unit economics—HELP ME turn the idea into a confirmed workload, a defensible model starting point, and a low/likely/high cost-per-completed-task range, SO I CAN decide what to prototype, budget, test, or stop before committing engineering time or provider spend.</x:v>
+      </x:c>
+      <x:c r="G20" s="34" t="str"/>
     </x:row>
     <x:row r="21" ht="88" customHeight="1">
-      <x:c r="A21" s="20"/>
+      <x:c r="A21" s="20" t="str"/>
       <x:c r="B21" s="20" t="str">
         <x:v>Workflow design</x:v>
       </x:c>
@@ -868,12 +864,12 @@
         <x:v>How does the workflow change when the agent is introduced? List the future process as text steps.</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>1. Start with the idea. 2. Choose guided intake, known usage, or a safe example. 3. Confirm work, risk, data, input size, result shape, primary steps, checker steps, and per-task ceiling. 4. Reject any output-token workload field. 5. Freeze workload, catalog, cost-contract, and rule versions. 6. Calculate low/likely/high cost per completed task from model-specific output/retry profiles. 7. Independently recompute all three scenarios. 8. Exclude candidates that fail capability, policy, evidence, or ceiling rules. 9. Run evaluation, audit, and governance. 10. Return the decision to the human.</x:v>
-      </x:c>
-      <x:c r="G21" s="26"/>
+        <x:v>1. Ask what the builder is considering building. 2. Route to guided intake, known usage, or a safe example. 3. Capture job, consequence, data boundary, every required format, usage, and result shape. 4. If primary/checker steps are unknown, propose a deterministic starting workflow and show it for confirmation. 5. Freeze the confirmed/assumed ledger. 6. Load the dated catalog and versioned rules. 7. Calculate model-specific low/likely/high cost per completed task. 8. Filter hard capability and policy constraints, then rank only eligible evidence-qualified candidates. 9. Freeze the result. 10. Run Cost Evaluation, Evaluation, Audit, and Governance without allowing any stage to mutate or waive the prior artifact. 11. Return PASS/WARN/REVIEW_REQUIRED/BLOCKED with rule IDs. 12. The human approves, edits/reruns, escalates, or records a permitted override.</x:v>
+      </x:c>
+      <x:c r="G21" s="26" t="str"/>
     </x:row>
     <x:row r="22" ht="88" customHeight="1">
-      <x:c r="A22" s="20"/>
+      <x:c r="A22" s="20" t="str"/>
       <x:c r="B22" s="20" t="str">
         <x:v>Agent behavior</x:v>
       </x:c>
@@ -887,12 +883,12 @@
         <x:v>What does the agent observe, reason about, produce, and check before handing work back?</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>The workflow observes the confirmed workload and provenance; applies deterministic estimation and eligibility; freezes the result; then the Cost Evaluation Specialist enforces COST-001 through COST-006 and recomputes the ledger without calling the estimator formula. Wider evaluation, audit, and governance follow. A failure blocks through GOV-009; heuristic behavior evidence remains visible through GOV-015. These are logical specialists inside one deterministic app, not autonomous LLM agents.</x:v>
-      </x:c>
-      <x:c r="G22" s="26"/>
+        <x:v>IMPLEMENTED ARCHITECTURE: one governed Decision Orchestrator with hard-bordered deterministic specialist stages—not several autonomous LLM agents. OBSERVE: Intake records the user job, risk, data boundary, every required format, usage, and result shape. DECIDE: a Workflow Architect rule suggests primary/checker steps when unknown; the Estimator/Selector applies versioned eligibility and cost rules. ACT: it produces a frozen recommendation and cost spread. CHECK: the separate Cost Evaluation Specialist independently recomputes the ledger, Evaluation tests eligibility, Audit checks hashes/versions, Governance applies absolute rules, and a human owns the final judgment. No LLM sits in the recommendation or approval path.</x:v>
+      </x:c>
+      <x:c r="G22" s="26" t="str"/>
     </x:row>
     <x:row r="23" ht="88" customHeight="1">
-      <x:c r="A23" s="20"/>
+      <x:c r="A23" s="20" t="str"/>
       <x:c r="B23" s="20" t="str">
         <x:v>Context</x:v>
       </x:c>
@@ -906,12 +902,12 @@
         <x:v>What information, examples, rules, files, or user inputs does the agent need to perform well?</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>Current workload inputs are the idea, work, consequence of error, data class, modality, regulated status, completed tasks per day, information going in, result shape, reusable input, primary AI steps, checker steps, and cost-per-completed-task ceiling. Output tokens and retry multipliers come from the selected model profile. System context includes dated prices, capability metadata, cost-contract version, formulas, eligibility rules, governance rules, and engine version.</x:v>
-      </x:c>
-      <x:c r="G23" s="26"/>
+        <x:v>User inputs: product idea, recurring job, consequence of error, data sensitivity, regulatory status, all required formats, traffic, information going in, desired result shape, reusable input, and optional affordability ceiling. Output tokens, retry rate, and attempted calls are not user-entered facts: they come from the selected model's versioned planning distribution. If primary/checker steps are unknown, a deterministic workflow rule recommends a visible starting architecture for user confirmation.</x:v>
+      </x:c>
+      <x:c r="G23" s="26" t="str"/>
     </x:row>
     <x:row r="24" ht="88" customHeight="1">
-      <x:c r="A24" s="20"/>
+      <x:c r="A24" s="20" t="str"/>
       <x:c r="B24" s="20" t="str">
         <x:v>Tools</x:v>
       </x:c>
@@ -925,12 +921,12 @@
         <x:v>What tools, files, systems, or mock actions will the prototype use? Text descriptions are enough.</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>The prototype uses prompt-first intake, a versioned model catalog, versioned cost contract and governance rules, model-specific output/retry distributions, deterministic cost-per-completed-task math, a separately implemented cost ledger, eligibility filters, fixed regression cases, governance dispositions, and a human decision gate. It does not run live provider workloads or claim the current behavior profiles are measured facts.</x:v>
-      </x:c>
-      <x:c r="G24" s="26"/>
+        <x:v>Implemented prototype tools: prompt-first intake; versioned JSON model catalog; versioned intake and governance rules; deterministic scenario/cost and eligibility engine; fixed evaluation cases; audit invariants; governance dispositions; deterministic decision brief; artifact hub. Purchasing, provisioning, production routing, and deployment authorization remain disabled.</x:v>
+      </x:c>
+      <x:c r="G24" s="26" t="str"/>
     </x:row>
     <x:row r="25" ht="88" customHeight="1">
-      <x:c r="A25" s="20"/>
+      <x:c r="A25" s="20" t="str"/>
       <x:c r="B25" s="20" t="str">
         <x:v>Memory</x:v>
       </x:c>
@@ -944,12 +940,12 @@
         <x:v>What should the agent remember, and what should it not remember?</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>Current behavior is no-save by default: the idea and workload remain in browser memory and disappear on refresh; no application database stores them. A future save option must be explicit and user-owned. Persist only normalized workload fields, versions, forecasts, findings, and the decision record. Never store API keys, secrets, raw proprietary prompts, protected health information, or unrelated conversation history. Provide clear-session, export, and deletion controls.</x:v>
-      </x:c>
-      <x:c r="G25" s="26"/>
+        <x:v>Persist the named project, structured workload assumptions, selected catalog version, candidate models, calculations, recommendation, decision status, and override reason. Do not retain secrets, API keys, proprietary source data, protected health information, raw unrelated conversations, or sensitive content copied from a production workload. Users must be able to edit or delete saved plans.</x:v>
+      </x:c>
+      <x:c r="G25" s="26" t="str"/>
     </x:row>
     <x:row r="26" ht="88" customHeight="1">
-      <x:c r="A26" s="20"/>
+      <x:c r="A26" s="20" t="str"/>
       <x:c r="B26" s="20" t="str">
         <x:v>Output</x:v>
       </x:c>
@@ -963,12 +959,12 @@
         <x:v>What should the agent produce so a human can review it quickly and confidently?</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>The current result shows assumptions, dated catalog and cost-contract versions, low/likely/high cost per completed task, secondary monthly volume context, model output/retry evidence, attempted calls per completed task, policy-eligible starting point, alternatives, exclusions, rule findings, and the human decision state. It separates published price facts from heuristic behavior profiles and missing tools, retrieval, storage, infrastructure, and review costs.</x:v>
-      </x:c>
-      <x:c r="G26" s="26"/>
+        <x:v>A reviewable decision brief containing: JTBD/workload summary; confirmed and recommended assumptions; catalog timestamp; required formats; suggested primary/checker architecture; eligible and excluded candidates; low/likely/high cost per completed task as the primary unit; planned-volume monthly context; recommended model; why it won; what would change the result; uncovered fees; governance status; and the human decision. A maximum cost is never invented: an optional spending ceiling only filters candidates when the user supplies one.</x:v>
+      </x:c>
+      <x:c r="G26" s="26" t="str"/>
     </x:row>
     <x:row r="27" ht="88" customHeight="1">
-      <x:c r="A27" s="20"/>
+      <x:c r="A27" s="20" t="str"/>
       <x:c r="B27" s="20" t="str">
         <x:v>Failure handling</x:v>
       </x:c>
@@ -982,12 +978,12 @@
         <x:v>What should happen when the agent is unsure, missing data, or facing a risky case?</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>Stop or block when required facts are missing, no candidate meets hard constraints, a needed price field is absent, the catalog is stale, a check fails, the workload is unsupported, or an agent loop exceeds the safety limit. Require human review for high-risk, regulated, sensitive, or unknown cases. Preserve the partial result and state the exact reason; do not turn uncertainty into a confident recommendation.</x:v>
-      </x:c>
-      <x:c r="G27" s="26"/>
+        <x:v>Stop and request clarification when required inputs are missing. Mark estimates incomplete when price fields or provider charges are unknown. Do not recommend a model when none meets hard constraints or evidence is insufficient. Require human review for high-risk or regulated workloads, sensitive data, materially consequential decisions, stale catalog data, contradictory rules, or attempted commercial bias. Preserve partial work and explain the blocker.</x:v>
+      </x:c>
+      <x:c r="G27" s="26" t="str"/>
     </x:row>
     <x:row r="28" ht="88" customHeight="1">
-      <x:c r="A28" s="20"/>
+      <x:c r="A28" s="20" t="str"/>
       <x:c r="B28" s="20" t="str">
         <x:v>Approval</x:v>
       </x:c>
@@ -1001,12 +997,12 @@
         <x:v>Where does the human approve, edit, reject, or escalate the agent's work?</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>After the calculation and rule findings are visible, the human reviews assumptions, price coverage, exclusions, alternatives, and risk. They can approve, edit and rerun, reject, escalate, or record a permitted override. The current decision state lasts only for the browser session; durable approval and override records are not implemented yet.</x:v>
-      </x:c>
-      <x:c r="G28" s="26"/>
+        <x:v>After calculations, eligibility filtering, and the grounded recommendation are displayed—but before the decision is finalized. The user reviews assumptions, sources, exclusions, cost drivers, alternatives, and risk flags; then approves, edits and reruns, selects an alternative with an override reason, rejects the result, or escalates to architecture/governance review.</x:v>
+      </x:c>
+      <x:c r="G28" s="26" t="str"/>
     </x:row>
     <x:row r="29" ht="88" customHeight="1">
-      <x:c r="A29" s="20"/>
+      <x:c r="A29" s="20" t="str"/>
       <x:c r="B29" s="20" t="str">
         <x:v>Evaluation</x:v>
       </x:c>
@@ -1020,9 +1016,9 @@
         <x:v>What cases will prove the agent works, respects boundaries, and handles edge cases?</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>Use controlled synthetic cases with known math and outcomes. Test forbidden output-token input, ordered model output/retry distributions, checker and retry inclusion, cost-per-completed-task ranking, deliberate ledger corruption, GOV-009 propagation, GOV-015 heuristic disclosure, same-input determinism, risk/data fail-closed rules, unsupported modality, stale pricing, loop limits, candidate-order invariance, and rendered-app smoke. Future live evaluation must measure distributions by task and model.</x:v>
-      </x:c>
-      <x:c r="G29" s="26"/>
+        <x:v>Use controlled synthetic cases with known cost math and expected rule outcomes. Test a normal text workload, a cheap-model-eligible classification task, a quality-sensitive reasoning task, unsupported modality, excessive agent loops, missing output estimate, stale price data, no eligible model, high-risk medical drafting, and an attempted sponsored-provider bias. Evaluate calculation accuracy, rule consistency, explanation grounding, boundary compliance, and human comprehension.</x:v>
+      </x:c>
+      <x:c r="G29" s="26" t="str"/>
     </x:row>
     <x:row r="30" ht="88" customHeight="1">
       <x:c r="A30" s="39" t="str">
@@ -1041,12 +1037,12 @@
         <x:v>What single end-to-end loop will the prototype prove?</x:v>
       </x:c>
       <x:c r="F30" s="37" t="str">
-        <x:v>Prove one complete planning loop: idea → explicit workload assumptions → model-owned behavior profile → low/likely/high cost per completed task → independent ledger match → policy-eligible starting point → alternatives and coverage gaps → governance → human decision. The prototype proves the controlled planning method; it does not prove the heuristic distributions are actual production behavior.</x:v>
-      </x:c>
-      <x:c r="G30" s="37"/>
+        <x:v>Enter one AI workload plan → identify missing constraints → compare sourced catalog facts across OpenAI, Google, and Anthropic → calculate low/expected/high cost → rank only candidates with shared evidence → explain the recommendation and tuning options → let the human approve or override → display a saved decision brief.</x:v>
+      </x:c>
+      <x:c r="G30" s="37" t="str"/>
     </x:row>
     <x:row r="31" ht="88" customHeight="1">
-      <x:c r="A31" s="20"/>
+      <x:c r="A31" s="20" t="str"/>
       <x:c r="B31" s="20" t="str">
         <x:v>Prototype</x:v>
       </x:c>
@@ -1060,12 +1056,12 @@
         <x:v>What will the user type, upload, click, or review in the prototype?</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>The user types an idea, chooses guided intake or known usage, reviews the workload, selects a result shape, confirms primary and checker steps, sets an optional per-task ceiling, runs the estimate, inspects the cost-per-completed-task spread and model behavior evidence, reviews the recommendation and alternatives, opens rule findings, changes a risk or cost driver, reruns, and records a session-level decision.</x:v>
-      </x:c>
-      <x:c r="G31" s="26"/>
+        <x:v>The user describes the idea in everyday language; selects job, risk, data boundary, regulatory status, and every required format; chooses a stage profile or supplies usage; selects the desired result shape; reviews a deterministic recommendation for primary/checker steps; and optionally supplies a hard affordability ceiling. The user does not enter output tokens. The builder reviews low/likely/high completed-task cost, exclusions, why the model won, what would change it, governance findings, and then approves, edits/reruns, escalates, or records a permitted override.</x:v>
+      </x:c>
+      <x:c r="G31" s="26" t="str"/>
     </x:row>
     <x:row r="32" ht="88" customHeight="1">
-      <x:c r="A32" s="20"/>
+      <x:c r="A32" s="20" t="str"/>
       <x:c r="B32" s="20" t="str">
         <x:v>Data</x:v>
       </x:c>
@@ -1079,12 +1075,12 @@
         <x:v>List the fake data files, sample records, policies, or examples used in the prototype.</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>Demo-safe inputs include a dated catalog snapshot built from official provider model and pricing pages for OpenAI, Google, and Anthropic; versioned intake and governance rules; fictional workload profiles; and deterministic regression fixtures. No provider key, live customer prompt, medical record, employer data, or proprietary idea is required. Published rates are planning inputs, not proof of an actual invoice.</x:v>
-      </x:c>
-      <x:c r="G32" s="26"/>
+        <x:v>Implemented demo-safe inputs: a versioned catalog containing dated published facts for three OpenAI, two Google Gemini, and three Anthropic Claude models; versioned intake, eligibility, and governance rules; deterministic cost scenarios; ten fictional evaluation cases; and a synthetic RAG customer-support workload used in the demo. No secret, customer, employer, medical, or proprietary data is required.</x:v>
+      </x:c>
+      <x:c r="G32" s="26" t="str"/>
     </x:row>
     <x:row r="33" ht="88" customHeight="1">
-      <x:c r="A33" s="20"/>
+      <x:c r="A33" s="20" t="str"/>
       <x:c r="B33" s="20" t="str">
         <x:v>Evaluation</x:v>
       </x:c>
@@ -1098,12 +1094,12 @@
         <x:v>List at least five test cases, including happy path, edge case, and boundary case.</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>1. Output-token field: COST-001 rejects it. 2. Same workload across tiers: output distributions differ by model. 3. Checker added: completed-task cost increases. 4. Higher retry scenario: attempted calls and cost increase. 5. One-cent ledger corruption: cost evaluation fails. 6. Failed cost evaluation: GOV-009 blocks. 7. Heuristic behavior profile: GOV-015 warns. 8. Same input twice: result and hash match. 9. Unknown/high-risk/unsupported/stale cases fail closed. 10. Candidate reorder does not change ranking. 11. Render smoke shows result shape and checker inputs without output-token input.</x:v>
-      </x:c>
-      <x:c r="G33" s="26"/>
+        <x:v>1. Same frozen input produces the same hash/result. 2. Output tokens supplied by a user are rejected. 3. Low/likely/high output and retry distributions remain ordered. 4. Checker steps/retries increase completed-task cost. 5. Corrupting the frozen estimate causes the independent cost specialist to fail and governance to block. 6. Text+image requirements remain conjunctive. 7. Unsupported text+audio blocks rather than silently dropping a format. 8. Unknown workflow steps receive a visible deterministic recommendation. 9. Classification/Low selects Luna, Product Analysis/Medium selects Terra, and Complex Reasoning/High selects Sol. 10. High-risk, unknown-data, stale-catalog, excessive-loop, no-eligible-model, and affordability-ceiling boundaries fail closed.</x:v>
+      </x:c>
+      <x:c r="G33" s="26" t="str"/>
     </x:row>
     <x:row r="34" ht="88" customHeight="1">
-      <x:c r="A34" s="20"/>
+      <x:c r="A34" s="20" t="str"/>
       <x:c r="B34" s="20" t="str">
         <x:v>Evaluation</x:v>
       </x:c>
@@ -1117,12 +1113,12 @@
         <x:v>What happened when you tested the agent? Where did it pass, fail, or need a human?</x:v>
       </x:c>
       <x:c r="F34" s="46" t="str">
-        <x:v>Observed release-candidate result on August 9, 2026: 15 automated checks passed and 0 failed. They cover COST-001 through COST-006, model-owned output profiles, retries and checker cost, independent three-scenario recomputation, deliberate corruption, governance propagation, deterministic math, fail-closed safety, stable ranking, and rendered-page smoke. The catalog audit also corrected OpenAI Luna and Terra price drift against official documentation. These are control tests, not measured provider behavior or cross-provider quality evaluation.</x:v>
-      </x:c>
-      <x:c r="G34" s="26"/>
+        <x:v>Observed release-candidate results on August 9, 2026: 18 automated tests passed and 0 failed; production build and lint passed. Evidence covers deterministic math, independent cost recomputation, output-token input rejection, model-specific output/retry distributions, checker cost, multi-format eligibility, unknown-step workflow recommendations, visible model-tier changes, high-risk/unknown-data review, stale-catalog and unsupported-format blocking, loop controls, affordability filtering, candidate-order invariance, and rendered-app smoke coverage. The estimator completed without any AI credential or model call.</x:v>
+      </x:c>
+      <x:c r="G34" s="26" t="str"/>
     </x:row>
     <x:row r="35" ht="88" customHeight="1">
-      <x:c r="A35" s="20"/>
+      <x:c r="A35" s="20" t="str"/>
       <x:c r="B35" s="20" t="str">
         <x:v>Iteration</x:v>
       </x:c>
@@ -1136,12 +1132,12 @@
         <x:v>What did you change after testing, and why?</x:v>
       </x:c>
       <x:c r="F35" s="46" t="str">
-        <x:v>Evaluation exposed a material defect: output tokens were treated as a user workload input, one call could hide retries and a checker, and monthly cost was the primary result. The correction removes that field, adds model-owned behavior distributions, separates primary and checker steps, ranks cost per completed task, adds an independent Cost Evaluation Specialist, and keeps unmeasured behavior visible through GOV-015.</x:v>
-      </x:c>
-      <x:c r="G35" s="26"/>
+        <x:v>Evaluation feedback showed that user-entered output tokens, fixed calls, and a single monthly number created false precision. The cost contract now forbids output-token input, assigns each model a low/likely/high output and retry distribution, includes primary and checker calls, and ranks by cost per completed task. Question 4 now accepts multiple formats. Unknown workflow steps trigger a visible deterministic architecture recommendation. The maximum-cost field is now an optional user-supplied spending ceiling, not an assumed answer. The interface also explains why Terra wins the default tier and which inputs switch the result to Luna, Sol, or a blocked state.</x:v>
+      </x:c>
+      <x:c r="G35" s="26" t="str"/>
     </x:row>
     <x:row r="36" ht="88" customHeight="1">
-      <x:c r="A36" s="20"/>
+      <x:c r="A36" s="20" t="str"/>
       <x:c r="B36" s="20" t="str">
         <x:v>Constraints</x:v>
       </x:c>
@@ -1155,12 +1151,12 @@
         <x:v>What does the prototype not do yet? Be honest and specific.</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>The prototype does not yet measure its output/retry profiles with repeated provider runs, refresh prices automatically, run shared provider quality workloads, reconcile invoices, include every tool or infrastructure fee, save decisions, export to a user-owned repository, or provide a tested clear-session/delete workflow. Published price fields are dated facts; output and retry distributions are planning heuristics. Monthly scale is a forecast, not actual spend.</x:v>
-      </x:c>
-      <x:c r="G36" s="26"/>
+        <x:v>This is one deterministic governed decision workflow with logical specialist stages; it is not a set of independently deployed autonomous LLM agents. It compares sourced catalog facts across OpenAI, Google, and Anthropic, but only the OpenAI heuristic policy baseline can enter ranking. It has not yet run repeated task-by-model live workloads, measured task success, p10/p50/p90 output, retry/checker rates, latency, or actual charged cost. It does not purchase access, route production traffic, persist user ideas, ingest secrets/protected data, reconcile billing, cover every provider fee, or approve regulated deployment. Its authority is limited to versioned inputs, published price facts, deterministic calculations, and policy disposition; a human remains accountable.</x:v>
+      </x:c>
+      <x:c r="G36" s="26" t="str"/>
     </x:row>
     <x:row r="37" ht="88" customHeight="1">
-      <x:c r="A37" s="20"/>
+      <x:c r="A37" s="20" t="str"/>
       <x:c r="B37" s="20" t="str">
         <x:v>Demo</x:v>
       </x:c>
@@ -1174,9 +1170,9 @@
         <x:v>Describe what the working prototype shows. A reviewer should understand the demo loop from this text.</x:v>
       </x:c>
       <x:c r="F37" s="46" t="str">
-        <x:v>The working correction begins with a plain-language idea and visible prompt box. The user reviews assumptions, chooses result shape instead of output tokens, confirms primary and checker steps, and sees low/likely/high cost per completed task plus secondary monthly scale. The page shows model output/retry evidence, the hard cost-contract status, policy-eligible OpenAI starting point, catalog-only Google and Anthropic comparisons, exclusions, and governance findings.</x:v>
-      </x:c>
-      <x:c r="G37" s="26"/>
+        <x:v>The working governed release candidate asks what the builder is considering building and offers guided, known-usage, and safe-example routes. The workload freeze captures job, risk, data/regulation, multiple required formats, traffic, input size, desired result shape, cache, and optional affordability ceiling. When steps are unknown, a deterministic rule recommends a visible primary/checker architecture. The result shows model-specific low/likely/high cost per completed task, why the eligible model won, what changes it, catalog-only alternatives, and uncovered fees. Cost Evaluation independently recomputes the frozen ledger; Evaluation, Audit, and Governance run before the Human Decision Gate. The estimator itself uses deterministic code and spends $0.00 in model tokens.</x:v>
+      </x:c>
+      <x:c r="G37" s="26" t="str"/>
     </x:row>
     <x:row r="38" ht="88" customHeight="1">
       <x:c r="A38" s="42" t="str">
@@ -1195,12 +1191,12 @@
         <x:v>Would you pilot this? What still needs to be true before launch?</x:v>
       </x:c>
       <x:c r="F38" s="40" t="str">
-        <x:v>GO for a controlled prototype demonstration and a small pilot using synthetic or non-sensitive planning inputs. NO-GO for regulated decisions, protected content, purchasing, or production routing. Before an external pilot: make privacy choices explicit, add clear-session and export/delete controls, validate first-time-user completion, establish reviewed catalog refresh, expand browser/accessibility tests, and define the data owner before any AWS persistence is enabled.</x:v>
-      </x:c>
-      <x:c r="G38" s="40"/>
+        <x:v>GO for a first-user release-candidate pilot using synthetic or non-sensitive planning assumptions: 18/18 automated checks, build, and lint pass. NO-GO for regulated production decisions, purchasing, automated routing, protected content, or claims of measured cross-provider quality. Before a broader alpha: run moderated first-time-user sessions, add accessible browser-flow regression, persist a deletable/append-only decision record, and replace heuristic profiles only after repeated task-by-model evidence clears defined sample and confidence thresholds.</x:v>
+      </x:c>
+      <x:c r="G38" s="40" t="str"/>
     </x:row>
     <x:row r="39" ht="88" customHeight="1">
-      <x:c r="A39" s="20"/>
+      <x:c r="A39" s="20" t="str"/>
       <x:c r="B39" s="20" t="str">
         <x:v>Risk</x:v>
       </x:c>
@@ -1214,12 +1210,12 @@
         <x:v>What data, compliance, trust, or misuse risks must be managed?</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>The main risks are stale or incomplete prices, misleading precision, unsupported capability claims, commercial bias, overreliance on a planning estimate, and users entering confidential ideas, secrets, proprietary material, or regulated data. Current control: workload content stays in browser state and is not sent to a model or application database. Required next controls: no-save default, clear-session action, local export, explicit consent before cloud save, encryption, tenant isolation, retention limits, deletion, audit logging without prompt content, and a user-owned repository export that never happens automatically.</x:v>
-      </x:c>
-      <x:c r="G39" s="26"/>
+        <x:v>Risks include stale or incorrect prices; fabricated model capabilities; misleading precision; poor model-fit recommendations; users entering secrets, proprietary data, or protected information; commercial bias; overreliance on generated explanations; and use of the result as deployment approval. Controls include minimal data collection, source timestamps, structured calculations, eligibility rules, visible uncertainty, human approval, audit history, deletion, and commercial disclosure.</x:v>
+      </x:c>
+      <x:c r="G39" s="26" t="str"/>
     </x:row>
     <x:row r="40" ht="88" customHeight="1">
-      <x:c r="A40" s="20"/>
+      <x:c r="A40" s="20" t="str"/>
       <x:c r="B40" s="20" t="str">
         <x:v>Operations</x:v>
       </x:c>
@@ -1233,12 +1229,12 @@
         <x:v>Who reviews agent output, handles escalations, and owns final decisions?</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>The human decision owner confirms workload assumptions and owns the final choice. The deterministic intake, estimate, evaluation, audit, and governance stages have separate responsibilities but currently run inside one engine. Architecture, security, privacy, procurement, finance, or domain specialists own escalations in their areas. The system never owns purchasing, deployment, risk acceptance, or regulated-use authorization.</x:v>
-      </x:c>
-      <x:c r="G40" s="26"/>
+        <x:v>The human decision owner confirms workload assumptions and owns the final judgment. Intake, Workflow Architecture, Estimation/Selection, Cost Evaluation, Audit, and Governance have hard-bordered contracts and cannot waive one another's findings. Architecture, security, privacy, procurement, or domain specialists own escalations in their areas. The system never owns purchase, deployment, risk acceptance, budget approval, or regulated-use authorization.</x:v>
+      </x:c>
+      <x:c r="G40" s="26" t="str"/>
     </x:row>
     <x:row r="41" ht="88" customHeight="1">
-      <x:c r="A41" s="20"/>
+      <x:c r="A41" s="20" t="str"/>
       <x:c r="B41" s="20" t="str">
         <x:v>Monitoring</x:v>
       </x:c>
@@ -1252,12 +1248,12 @@
         <x:v>What would you monitor after launch to catch drift, failures, or bad outcomes?</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>Monitor catalog age and price-source changes; cost-contract failures; output-token rejection attempts; predicted versus measured output and retry distributions; completed-task success; checker use; cost per completed task; calculation and rule failures; time to estimate; assumptions; review/block reasons; unsupported workloads; per-task ceiling variance; and documentation drift. After persistence exists, compare forecasts with provider usage and invoices without storing prompt content.</x:v>
-      </x:c>
-      <x:c r="G41" s="26"/>
+        <x:v>Monitor catalog freshness and failed refreshes; estimate versus actual usage and cost; calculation errors; recommendation and override rates; no-eligible-model frequency; stale-data warnings; explanation-to-structured-result consistency; user-reported incorrect capability claims; high-risk escalations; sensitive-data attempts; latency; task completion; and whether recommended models continue to pass representative evaluations.</x:v>
+      </x:c>
+      <x:c r="G41" s="26" t="str"/>
     </x:row>
     <x:row r="42" ht="88" customHeight="1">
-      <x:c r="A42" s="20"/>
+      <x:c r="A42" s="20" t="str"/>
       <x:c r="B42" s="20" t="str">
         <x:v>Feedback</x:v>
       </x:c>
@@ -1271,12 +1267,12 @@
         <x:v>How would you collect feedback and decide what to improve next?</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>After each planning session ask whether the result was understandable, useful, trusted, and actionable. Capture what the user changed or rejected and why. Observe first-time builders completing the flow without coaching. Review failures and escalations weekly. Prioritize by decision harm, frequency, user impact, and evidence—not by the loudest feature request.</x:v>
-      </x:c>
-      <x:c r="G42" s="26"/>
+        <x:v>After each decision brief, ask whether the recommendation was understandable, useful, trusted, and acted on; capture the reason for overrides; interview pilot users about missing criteria and research time; compare estimates with actual usage when available; review failure and escalation cases weekly; and prioritize changes by decision harm, frequency, user impact, and evidence—not by feature requests alone.</x:v>
+      </x:c>
+      <x:c r="G42" s="26" t="str"/>
     </x:row>
     <x:row r="43" ht="88" customHeight="1">
-      <x:c r="A43" s="20"/>
+      <x:c r="A43" s="20" t="str"/>
       <x:c r="B43" s="20" t="str">
         <x:v>Rollout</x:v>
       </x:c>
@@ -1290,17 +1286,17 @@
         <x:v>What is the smallest safe launch or pilot path?</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>Start with three recorded sessions using fictional or non-sensitive workloads, including one high-risk case, one stale or unsupported case, and one normal planning case. Then invite three to five first-time AI product builders. Keep no-save as the default. Test local export and clear-session before cloud persistence. Only after privacy and ownership controls pass should a small AWS-backed history pilot begin; shared Google and Anthropic evaluation comes later with user-owned keys, synthetic cases, and a hard run budget.</x:v>
-      </x:c>
-      <x:c r="G43" s="26"/>
+        <x:v>Begin with one product builder and synthetic or non-sensitive workloads using the three-provider catalog. Run three real planning sessions plus high-risk, stale-catalog, unsupported multi-format, and recommendation-switch demos. Then invite three to five first-time builders with fictional or sanitized plans. Connect OpenAI, Google Gemini, and Anthropic Claude to shared live evaluation only after protected provider keys, a per-run budget cap, synthetic workload suite, adapters, blinded scoring, source/freshness controls, and promotion thresholds pass.</x:v>
+      </x:c>
+      <x:c r="G43" s="26" t="str"/>
     </x:row>
     <x:row r="44" ht="88" customHeight="1">
-      <x:c r="A44" s="20"/>
+      <x:c r="A44" s="20" t="str"/>
       <x:c r="B44" s="20" t="str">
         <x:v>Communication</x:v>
       </x:c>
       <x:c r="C44" s="20" t="str">
-        <x:v>4-minute video outline</x:v>
+        <x:v>2–3 minute video outline</x:v>
       </x:c>
       <x:c r="D44" s="20" t="str">
         <x:v>Executive product review</x:v>
@@ -1309,9 +1305,9 @@
         <x:v>How will your video cover intro, problem, discovery, solution demo, eval rigor, impact, and launch plan?</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>0:00–0:30 Open with false precision in model cost. 0:30–1:00 Introduce the first user and product. 1:00–1:35 Show the idea-first intake. 1:35–2:20 Show result shape, model-owned output/retry distribution, primary and checker steps, and cost per completed task. 2:20–3:05 Show the independent Cost Evaluation Specialist, COST-001 through COST-006, GOV-009 block, and GOV-015 warning. 3:05–3:35 State 15/15 evidence and limits. 3:35–4:00 close on measured distributions, privacy controls, and the human decision.</x:v>
-      </x:c>
-      <x:c r="G44" s="26"/>
+        <x:v>0:00–0:20 Hook: Pick the right model; know the cost. 0:20–0:45 Persona, JTBD, and the false-precision problem. 0:45–1:20 Demo prompt-first intake, multi-format selection, recommended workflow steps, and optional ceiling. 1:20–1:50 Show cost per completed task, the Luna/Terra/Sol tier switch, and catalog-only providers. 1:50–2:15 Explain one Decision Orchestrator plus deterministic specialist checks and the human gate. 2:15–2:40 State 18/18 evidence and current limits. 2:40–3:00 Explain the next measured synthetic evaluation and promotion threshold.</x:v>
+      </x:c>
+      <x:c r="G44" s="26" t="str"/>
     </x:row>
     <x:row r="45" ht="88" customHeight="1">
       <x:c r="A45" s="45" t="str">
@@ -1330,12 +1326,12 @@
         <x:v>Is every grading-critical decision written directly in this sheet with no required link-outs?</x:v>
       </x:c>
       <x:c r="F45" s="47" t="str">
-        <x:v>YES. Every grading-critical decision is written in this sheet: user, workflow, trigger, current process, problem, agent opportunity, safe data, human boundary, success metric, demo, design, tools, memory, output, failure handling, approval, eval plan and results, iteration, limitations, readiness, privacy, operating model, monitoring, feedback, pilot, and video plan. No external link is required to understand the work.</x:v>
-      </x:c>
-      <x:c r="G45" s="43"/>
+        <x:v>YES. Discovery, persona, JTBD, problem, agent opportunity, implemented single-orchestrator architecture, specialist boundaries, tools, memory, failure rules, human checkpoint, observed 18/18 evaluation evidence, iteration, working-demo behavior, limitations, readiness, monitoring, feedback, rollout, and video story are written directly in this sheet.</x:v>
+      </x:c>
+      <x:c r="G45" s="43" t="str"/>
     </x:row>
     <x:row r="46" ht="88" customHeight="1">
-      <x:c r="A46" s="20"/>
+      <x:c r="A46" s="20" t="str"/>
       <x:c r="B46" s="20" t="str">
         <x:v>Submission</x:v>
       </x:c>
@@ -1349,12 +1345,12 @@
         <x:v>Can a reviewer understand the working prototype loop from the PRD and video?</x:v>
       </x:c>
       <x:c r="F46" s="46" t="str">
-        <x:v>YES. A reviewer can follow the corrected loop directly from this PRD and four-minute video: idea → confirmed workload without output-token input → model-owned distribution → cost per completed task → independent cost evaluation → policy eligibility → governance → human decision. The PRD states that current behavior profiles are heuristics and requires same-commit deployment evidence before submission.</x:v>
-      </x:c>
-      <x:c r="G46" s="26"/>
+        <x:v>YES. The prompt-first routes, multi-format workload freeze, workflow-step recommendation, model-specific output/retry distributions, cost per completed task, eligibility filtering, Luna/Terra/Sol switch, separate hard checks, Human Decision Gate, and measured-evaluation next step are described directly above. The prototype is correctly labeled as one governed deterministic decision workflow—not autonomous multi-agent deployment.</x:v>
+      </x:c>
+      <x:c r="G46" s="26" t="str"/>
     </x:row>
     <x:row r="47" ht="88" customHeight="1">
-      <x:c r="A47" s="21"/>
+      <x:c r="A47" s="21" t="str"/>
       <x:c r="B47" s="21" t="str">
         <x:v>Submission</x:v>
       </x:c>
@@ -1362,15 +1358,15 @@
         <x:v>Video check</x:v>
       </x:c>
       <x:c r="D47" s="21" t="str">
-        <x:v>Four-minute story</x:v>
+        <x:v>Two-to-three-minute story</x:v>
       </x:c>
       <x:c r="E47" s="30" t="str">
-        <x:v>Does the 4-minute video show the product clearly, concisely, and persuasively?</x:v>
+        <x:v>Does the 2–3 minute video show the product clearly, concisely, and persuasively?</x:v>
       </x:c>
       <x:c r="F47" s="48" t="str">
-        <x:v>RECORDING-READY RELEASE CANDIDATE. The eight-slide deck and four-minute talk track cover the problem, first user, corrected cost model, independent Cost Evaluation Specialist, 15/15 evidence, heuristic limits, and measured-evaluation next step. Before submission, verify COST-001 and GOV-015 on the live page, run one clean rehearsal, and keep every spoken claim aligned with this PRD.</x:v>
-      </x:c>
-      <x:c r="G47" s="27"/>
+        <x:v>READY TO RECORD. A timed 2:30 script and operator checklist are complete. Before submission, record it, verify runtime, confirm the high-risk review state is visible, and check that the narration matches the PRD, evaluation, limitations, three-provider catalog, and shared-evaluation next step.</x:v>
+      </x:c>
+      <x:c r="G47" s="27" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Align PRD controls with faculty feedback
</commit_message>
<xml_diff>
--- a/artifacts/AI_Build_Crew_Agentic_AI_PRD_COST_CONTRACT.xlsx
+++ b/artifacts/AI_Build_Crew_Agentic_AI_PRD_COST_CONTRACT.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R4cefe2b729024d87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R8f776e9429034f61"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -805,7 +805,7 @@
         <x:v>What is one practical metric that would show the agent is useful?</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>Primary metric: a first-time builder can produce a first estimate in under three minutes and explain the recommendation, one cost assumption, and one alternative tradeoff. Release quality requires every deterministic cost, evaluation, audit, and governance regression case to pass; high-risk, unknown-safety, or unsupported multi-format work can never be marked ready without review.</x:v>
+        <x:v>PRIMARY ACCURACY METRIC: 100% of controlled cost cases must match the known answer key to the engine's eight-decimal precision; any mismatch blocks release. SAFETY METRIC: zero fabricated price/capability claims and zero high-risk, unknown-safety, or unsupported multi-format cases marked ready. SECONDARY USABILITY TARGET: a first-time builder produces an estimate in under three minutes and can explain one assumption and one alternative tradeoff.</x:v>
       </x:c>
       <x:c r="G18" s="26" t="str"/>
     </x:row>
@@ -864,7 +864,7 @@
         <x:v>How does the workflow change when the agent is introduced? List the future process as text steps.</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>1. Ask what the builder is considering building. 2. Route to guided intake, known usage, or a safe example. 3. Capture job, consequence, data boundary, every required format, usage, and result shape. 4. If primary/checker steps are unknown, propose a deterministic starting workflow and show it for confirmation. 5. Freeze the confirmed/assumed ledger. 6. Load the dated catalog and versioned rules. 7. Calculate model-specific low/likely/high cost per completed task. 8. Filter hard capability and policy constraints, then rank only eligible evidence-qualified candidates. 9. Freeze the result. 10. Run Cost Evaluation, Evaluation, Audit, and Governance without allowing any stage to mutate or waive the prior artifact. 11. Return PASS/WARN/REVIEW_REQUIRED/BLOCKED with rule IDs. 12. The human approves, edits/reruns, escalates, or records a permitted override.</x:v>
+        <x:v>1. Ask what the builder is considering building. 2. Route to guided intake, known usage, or a safe example. 3. Capture job, consequence, data boundary, every required format, usage, and result shape. 4. If primary/checker steps are unknown, propose a deterministic starting workflow and show it for confirmation. 5. Freeze the confirmed/assumed ledger. 6. Load the dated catalog and versioned rules. 7. Calculate model-specific low/likely/high cost per completed task. 8. Apply the visible rubric: capability, context, format, freshness, risk, regulation, and minimum quality are pass/fail gates; among surviving evaluated candidates, likely cost per completed task has 100% ranking weight. Latency and quality above the threshold have 0% weight until measured. 9. Freeze the result. 10. Run Cost Evaluation, Evaluation, Audit, and Governance without allowing any stage to mutate or waive the prior artifact. 11. Return PASS/WARN/REVIEW_REQUIRED/BLOCKED with rule IDs. 12. The human approves, edits/reruns, escalates, or records a permitted override.</x:v>
       </x:c>
       <x:c r="G21" s="26" t="str"/>
     </x:row>
@@ -1248,7 +1248,7 @@
         <x:v>What would you monitor after launch to catch drift, failures, or bad outcomes?</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>Monitor catalog freshness and failed refreshes; estimate versus actual usage and cost; calculation errors; recommendation and override rates; no-eligible-model frequency; stale-data warnings; explanation-to-structured-result consistency; user-reported incorrect capability claims; high-risk escalations; sensitive-data attempts; latency; task completion; and whether recommended models continue to pass representative evaluations.</x:v>
+        <x:v>Two hard stop thresholds lead the operating dashboard. 1. CALCULATION ACCURACY: any controlled-case mismatch against the known answer key blocks release and returns to the earliest failed cost stage. After actual-charge integration, an absolute forecast variance above 20% across the first 30 comparable completed tasks pauses profile promotion and triggers recalibration. 2. FABRICATED CAPABILITY OR PRICE: target zero; one confirmed occurrence blocks the candidate catalog and rolls back to the last-known-good snapshot. Catalog age beyond its freshness limit also blocks. Rollback restores the prior immutable release/Sites version, preserves the failed evidence, and uses a normal Git revert rather than moving a tag.</x:v>
       </x:c>
       <x:c r="G41" s="26" t="str"/>
     </x:row>

</xml_diff>